<commit_message>
Have further cleaned the Brewers Friend data to be totally compliant with BJCP 2021.
</commit_message>
<xml_diff>
--- a/BJCP_update_Style_Name.xlsx
+++ b/BJCP_update_Style_Name.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28715"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{E1A2B7B5-9E33-431D-A9EC-BE7704FB16A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EDF806C6-4199-4D00-8160-C65B4015DC94}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8CD16EC4-7D92-4926-8059-7F57245932E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="106">
   <si>
     <t>Style</t>
   </si>
@@ -340,6 +340,15 @@
   </si>
   <si>
     <t>27B</t>
+  </si>
+  <si>
+    <t>Premium American Lager</t>
+  </si>
+  <si>
+    <t>American Lager</t>
+  </si>
+  <si>
+    <t>1B</t>
   </si>
 </sst>
 </file>
@@ -711,7 +720,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B058E539-E1CD-4261-A2CD-DF658B9C05DC}">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.140625" customWidth="1"/>
@@ -1148,6 +1157,17 @@
         <v>102</v>
       </c>
     </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>103</v>
+      </c>
+      <c r="B40" t="s">
+        <v>104</v>
+      </c>
+      <c r="C40" t="s">
+        <v>105</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>